<commit_message>
feat: update reinspection suite, pptx generator, annotator, assets and latest datasets
</commit_message>
<xml_diff>
--- a/Color_Template.xlsx
+++ b/Color_Template.xlsx
@@ -100,7 +100,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="151">
+  <fills count="153">
     <fill>
       <patternFill/>
     </fill>
@@ -999,6 +999,18 @@
       <patternFill patternType="solid">
         <fgColor rgb="FF803939"/>
         <bgColor rgb="FF803939"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF80252F"/>
+        <bgColor rgb="FF80252F"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF698011"/>
+        <bgColor rgb="FF698011"/>
       </patternFill>
     </fill>
   </fills>
@@ -1101,7 +1113,7 @@
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="181">
+  <cellXfs count="183">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1635,6 +1647,8 @@
     <xf numFmtId="0" fontId="0" fillId="149" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="151" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="152" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2331,7 +2345,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="C3:M63"/>
+  <dimension ref="C3:M65"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.90625" defaultRowHeight="13.85"/>
   <cols>
     <col width="11.54296875" customWidth="1" style="92" min="1" max="1"/>
@@ -3701,7 +3715,50 @@
         </is>
       </c>
     </row>
-    <row r="64" ht="20" customHeight="1" s="92"/>
+    <row r="64" ht="20" customHeight="1" s="92">
+      <c r="C64" s="163" t="inlineStr">
+        <is>
+          <t>Lacing</t>
+        </is>
+      </c>
+      <c r="D64" s="181" t="n"/>
+      <c r="E64" s="165" t="n">
+        <v>128</v>
+      </c>
+      <c r="F64" s="165" t="n">
+        <v>37</v>
+      </c>
+      <c r="G64" s="165" t="n">
+        <v>47</v>
+      </c>
+      <c r="H64" s="166" t="inlineStr">
+        <is>
+          <t>80252F</t>
+        </is>
+      </c>
+    </row>
+    <row r="65" ht="20" customHeight="1" s="92">
+      <c r="C65" s="163" t="inlineStr">
+        <is>
+          <t>Shoe lace length</t>
+        </is>
+      </c>
+      <c r="D65" s="182" t="n"/>
+      <c r="E65" s="165" t="n">
+        <v>105</v>
+      </c>
+      <c r="F65" s="165" t="n">
+        <v>128</v>
+      </c>
+      <c r="G65" s="165" t="n">
+        <v>17</v>
+      </c>
+      <c r="H65" s="166" t="inlineStr">
+        <is>
+          <t>698011</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="C3:H3"/>

</xml_diff>

<commit_message>
feat(pptx): enhance chart scaling, pie labels, visual annotations, and update spec
</commit_message>
<xml_diff>
--- a/Color_Template.xlsx
+++ b/Color_Template.xlsx
@@ -100,7 +100,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="153">
+  <fills count="157">
     <fill>
       <patternFill/>
     </fill>
@@ -1011,6 +1011,30 @@
       <patternFill patternType="solid">
         <fgColor rgb="FF698011"/>
         <bgColor rgb="FF698011"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFAC5C95"/>
+        <bgColor rgb="FFAC5C95"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF953735"/>
+        <bgColor rgb="FF953735"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC3D4EF"/>
+        <bgColor rgb="FFC3D4EF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF403152"/>
+        <bgColor rgb="FF403152"/>
       </patternFill>
     </fill>
   </fills>
@@ -1113,7 +1137,7 @@
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="183">
+  <cellXfs count="191">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1649,6 +1673,30 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="151" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="152" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="153" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="154" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="155" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="156" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2683,19 +2731,19 @@
           <t>Components inconsistent</t>
         </is>
       </c>
-      <c r="D17" s="110" t="n"/>
-      <c r="E17" s="96" t="n">
-        <v>102</v>
-      </c>
-      <c r="F17" s="96" t="n">
-        <v>153</v>
-      </c>
-      <c r="G17" s="96" t="n">
-        <v>255</v>
-      </c>
-      <c r="H17" s="111" t="inlineStr">
-        <is>
-          <t>6699FF</t>
+      <c r="D17" s="183" t="n"/>
+      <c r="E17" s="184" t="n">
+        <v>172</v>
+      </c>
+      <c r="F17" s="184" t="n">
+        <v>92</v>
+      </c>
+      <c r="G17" s="184" t="n">
+        <v>149</v>
+      </c>
+      <c r="H17" s="185" t="inlineStr">
+        <is>
+          <t>AC5C95</t>
         </is>
       </c>
     </row>
@@ -3212,19 +3260,19 @@
           <t>Over buffing</t>
         </is>
       </c>
-      <c r="D41" s="138" t="n"/>
-      <c r="E41" s="114" t="n">
-        <v>14</v>
-      </c>
-      <c r="F41" s="114" t="n">
-        <v>141</v>
-      </c>
-      <c r="G41" s="114" t="n">
-        <v>135</v>
-      </c>
-      <c r="H41" s="97" t="inlineStr">
-        <is>
-          <t>0E8D87</t>
+      <c r="D41" s="186" t="n"/>
+      <c r="E41" s="187" t="n">
+        <v>149</v>
+      </c>
+      <c r="F41" s="187" t="n">
+        <v>55</v>
+      </c>
+      <c r="G41" s="187" t="n">
+        <v>53</v>
+      </c>
+      <c r="H41" s="188" t="inlineStr">
+        <is>
+          <t>953735</t>
         </is>
       </c>
     </row>
@@ -3346,19 +3394,19 @@
           <t>Sole attachment</t>
         </is>
       </c>
-      <c r="D47" s="145" t="n"/>
-      <c r="E47" s="96" t="n">
-        <v>112</v>
-      </c>
-      <c r="F47" s="96" t="n">
-        <v>48</v>
-      </c>
-      <c r="G47" s="96" t="n">
-        <v>160</v>
-      </c>
-      <c r="H47" s="97" t="inlineStr">
-        <is>
-          <t>7030A0</t>
+      <c r="D47" s="189" t="n"/>
+      <c r="E47" s="184" t="n">
+        <v>195</v>
+      </c>
+      <c r="F47" s="184" t="n">
+        <v>212</v>
+      </c>
+      <c r="G47" s="184" t="n">
+        <v>239</v>
+      </c>
+      <c r="H47" s="188" t="inlineStr">
+        <is>
+          <t>C3D4EF</t>
         </is>
       </c>
     </row>
@@ -3479,19 +3527,19 @@
           <t>Toe off center</t>
         </is>
       </c>
-      <c r="D53" s="151" t="n"/>
-      <c r="E53" s="96" t="n">
-        <v>6</v>
-      </c>
-      <c r="F53" s="96" t="n">
-        <v>38</v>
-      </c>
-      <c r="G53" s="96" t="n">
-        <v>208</v>
-      </c>
-      <c r="H53" s="97" t="inlineStr">
-        <is>
-          <t>0626D0</t>
+      <c r="D53" s="190" t="n"/>
+      <c r="E53" s="184" t="n">
+        <v>64</v>
+      </c>
+      <c r="F53" s="184" t="n">
+        <v>49</v>
+      </c>
+      <c r="G53" s="184" t="n">
+        <v>82</v>
+      </c>
+      <c r="H53" s="188" t="inlineStr">
+        <is>
+          <t>403152</t>
         </is>
       </c>
     </row>

</xml_diff>